<commit_message>
Criando lógica de unidade
</commit_message>
<xml_diff>
--- a/Base_RAs/022__alunos_com_informacao_de_parceria_2026-07-27T16_00_39.4344432-04_00.xlsx
+++ b/Base_RAs/022__alunos_com_informacao_de_parceria_2026-07-27T16_00_39.4344432-04_00.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://senaimt-my.sharepoint.com/personal/manoel_campos_sfiemt_ind_br/Documents/Área de Trabalho/AutomatizacaoERP/Base_RAs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="51" documentId="8_{707DEA74-B68B-4E6A-B857-F924FB2D3DDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F4134AC5-0D29-48A5-88E9-FBC8F26C7CC1}"/>
+  <xr:revisionPtr revIDLastSave="57" documentId="8_{707DEA74-B68B-4E6A-B857-F924FB2D3DDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5877BEBF-4739-45F3-88E6-2F67B9C4A0D6}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="2685" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="2685" windowWidth="24240" windowHeight="13020" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resultado da consulta" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8698" uniqueCount="3527">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8711" uniqueCount="3527">
   <si>
     <t>CodFilialSGE</t>
   </si>
@@ -12835,7 +12835,7 @@
       <c r="H45" t="s">
         <v>1386</v>
       </c>
-      <c r="I45" t="s">
+      <c r="I45" s="3" t="s">
         <v>1387</v>
       </c>
       <c r="J45" s="1">
@@ -46500,48 +46500,63 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36902C53-BC33-4603-BFD3-82F285A025AB}">
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="32.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="35.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="58.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="1">
-        <v>1</v>
+      <c r="A1" t="s">
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>109</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>110</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>305</v>
+        <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>306</v>
+        <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>307</v>
+        <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>308</v>
-      </c>
-      <c r="J1" s="1">
-        <v>1</v>
-      </c>
-      <c r="K1" s="1">
-        <v>2</v>
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
       </c>
       <c r="L1" t="s">
-        <v>115</v>
+        <v>11</v>
       </c>
       <c r="M1" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -46555,22 +46570,22 @@
         <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>828</v>
+        <v>110</v>
       </c>
       <c r="E2" t="s">
-        <v>829</v>
+        <v>305</v>
       </c>
       <c r="F2" t="s">
         <v>17</v>
       </c>
       <c r="G2" t="s">
-        <v>830</v>
+        <v>306</v>
       </c>
       <c r="H2" t="s">
-        <v>831</v>
+        <v>307</v>
       </c>
       <c r="I2" t="s">
-        <v>832</v>
+        <v>308</v>
       </c>
       <c r="J2" s="1">
         <v>1</v>
@@ -46579,7 +46594,7 @@
         <v>2</v>
       </c>
       <c r="L2" t="s">
-        <v>833</v>
+        <v>115</v>
       </c>
       <c r="M2" t="s">
         <v>22</v>
@@ -46596,22 +46611,22 @@
         <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>110</v>
+        <v>828</v>
       </c>
       <c r="E3" t="s">
-        <v>3208</v>
+        <v>829</v>
       </c>
       <c r="F3" t="s">
         <v>17</v>
       </c>
       <c r="G3" t="s">
-        <v>3209</v>
+        <v>830</v>
       </c>
       <c r="H3" t="s">
-        <v>3210</v>
+        <v>831</v>
       </c>
       <c r="I3" t="s">
-        <v>3211</v>
+        <v>832</v>
       </c>
       <c r="J3" s="1">
         <v>1</v>
@@ -46620,7 +46635,7 @@
         <v>2</v>
       </c>
       <c r="L3" t="s">
-        <v>115</v>
+        <v>833</v>
       </c>
       <c r="M3" t="s">
         <v>22</v>
@@ -46637,22 +46652,22 @@
         <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>828</v>
+        <v>110</v>
       </c>
       <c r="E4" t="s">
-        <v>3400</v>
+        <v>3208</v>
       </c>
       <c r="F4" t="s">
         <v>17</v>
       </c>
       <c r="G4" t="s">
-        <v>3401</v>
+        <v>3209</v>
       </c>
       <c r="H4" t="s">
-        <v>3402</v>
+        <v>3210</v>
       </c>
       <c r="I4" t="s">
-        <v>3403</v>
+        <v>3211</v>
       </c>
       <c r="J4" s="1">
         <v>1</v>
@@ -46661,7 +46676,7 @@
         <v>2</v>
       </c>
       <c r="L4" t="s">
-        <v>833</v>
+        <v>115</v>
       </c>
       <c r="M4" t="s">
         <v>22</v>
@@ -46678,22 +46693,22 @@
         <v>14</v>
       </c>
       <c r="D5" t="s">
-        <v>3505</v>
+        <v>828</v>
       </c>
       <c r="E5" t="s">
-        <v>3506</v>
+        <v>3400</v>
       </c>
       <c r="F5" t="s">
         <v>17</v>
       </c>
       <c r="G5" t="s">
-        <v>3507</v>
+        <v>3401</v>
       </c>
       <c r="H5" t="s">
-        <v>3508</v>
+        <v>3402</v>
       </c>
       <c r="I5" t="s">
-        <v>3509</v>
+        <v>3403</v>
       </c>
       <c r="J5" s="1">
         <v>1</v>
@@ -46702,9 +46717,50 @@
         <v>2</v>
       </c>
       <c r="L5" t="s">
+        <v>833</v>
+      </c>
+      <c r="M5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>1</v>
+      </c>
+      <c r="B6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" t="s">
+        <v>3505</v>
+      </c>
+      <c r="E6" t="s">
+        <v>3506</v>
+      </c>
+      <c r="F6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" t="s">
+        <v>3507</v>
+      </c>
+      <c r="H6" t="s">
+        <v>3508</v>
+      </c>
+      <c r="I6" t="s">
+        <v>3509</v>
+      </c>
+      <c r="J6" s="1">
+        <v>1</v>
+      </c>
+      <c r="K6" s="1">
+        <v>2</v>
+      </c>
+      <c r="L6" t="s">
         <v>3510</v>
       </c>
-      <c r="M5" t="s">
+      <c r="M6" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>